<commit_message>
Fix family member part-of-speech mapping
</commit_message>
<xml_diff>
--- a/Module_E_2027_Vocabulary_Master.xlsx
+++ b/Module_E_2027_Vocabulary_Master.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rda8bd8cbb23a4611"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vocabulary" sheetId="2" r:id="R6231e23f850b4aaa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R2a592ad3d3584251"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vocabulary" sheetId="2" r:id="Re82d665f084c47b2"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -723,7 +723,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfed7af74aca0491f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re3c161ffeafc491f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2558,8 +2558,8 @@
 developed</x:v>
       </x:c>
       <x:c r="P40" s="16" t="str">
-        <x:v>Adj Adj
-Adj Adj</x:v>
+        <x:v>Adjective
+Adjective</x:v>
       </x:c>
     </x:row>
     <x:row r="41" ht="36" customHeight="1">
@@ -3476,8 +3476,8 @@
 investment</x:v>
       </x:c>
       <x:c r="P60" s="16" t="str">
-        <x:v>N N
-N N</x:v>
+        <x:v>Noun
+Noun</x:v>
       </x:c>
     </x:row>
     <x:row r="61" ht="36" customHeight="1">
@@ -3747,8 +3747,8 @@
 concerned with sth</x:v>
       </x:c>
       <x:c r="P66" s="16" t="str">
-        <x:v>Adj Prep
-Adj Prep
+        <x:v>Adjective
+Preposition
 Phrase</x:v>
       </x:c>
     </x:row>
@@ -4698,8 +4698,8 @@
 significance</x:v>
       </x:c>
       <x:c r="P87" s="16" t="str">
-        <x:v>Adv N
-Adv N</x:v>
+        <x:v>Adverb
+Noun</x:v>
       </x:c>
     </x:row>
     <x:row r="88" ht="36" customHeight="1">
@@ -5972,8 +5972,8 @@
 specify</x:v>
       </x:c>
       <x:c r="P115" s="16" t="str">
-        <x:v>Adv V
-Adv V</x:v>
+        <x:v>Adverb
+Verb</x:v>
       </x:c>
     </x:row>
     <x:row r="116" ht="36" customHeight="1">
@@ -6198,8 +6198,8 @@
 psychologist</x:v>
       </x:c>
       <x:c r="P120" s="16" t="str">
-        <x:v>Adj N
-Adj N</x:v>
+        <x:v>Adjective
+Noun</x:v>
       </x:c>
     </x:row>
     <x:row r="121" ht="36" customHeight="1">
@@ -6248,8 +6248,8 @@
 participation</x:v>
       </x:c>
       <x:c r="P121" s="16" t="str">
-        <x:v>N N
-N N</x:v>
+        <x:v>Noun
+Noun</x:v>
       </x:c>
     </x:row>
     <x:row r="122" ht="36" customHeight="1">
@@ -6434,8 +6434,8 @@
 existing</x:v>
       </x:c>
       <x:c r="P125" s="16" t="str">
-        <x:v>N Adj
-N Adj</x:v>
+        <x:v>Noun
+Adjective</x:v>
       </x:c>
     </x:row>
     <x:row r="126" ht="36" customHeight="1">
@@ -7328,8 +7328,8 @@
 educator</x:v>
       </x:c>
       <x:c r="P145" s="16" t="str">
-        <x:v>Adj N
-Adj N</x:v>
+        <x:v>Adjective
+Noun</x:v>
       </x:c>
     </x:row>
     <x:row r="146" ht="36" customHeight="1">
@@ -9002,8 +9002,8 @@
 investigator</x:v>
       </x:c>
       <x:c r="P182" s="16" t="str">
-        <x:v>N N
-N N</x:v>
+        <x:v>Noun
+Noun</x:v>
       </x:c>
     </x:row>
     <x:row r="183" ht="36" customHeight="1">
@@ -9768,8 +9768,8 @@
 analyst</x:v>
       </x:c>
       <x:c r="P199" s="16" t="str">
-        <x:v>V N
-V N</x:v>
+        <x:v>Verb
+Noun</x:v>
       </x:c>
     </x:row>
     <x:row r="200" ht="36" customHeight="1">
@@ -9950,8 +9950,8 @@
 regarding</x:v>
       </x:c>
       <x:c r="P203" s="16" t="str">
-        <x:v>Adv Prep
-Adv Prep</x:v>
+        <x:v>Adverb
+Preposition</x:v>
       </x:c>
     </x:row>
     <x:row r="204" ht="36" customHeight="1">
@@ -10680,8 +10680,8 @@
 criticism</x:v>
       </x:c>
       <x:c r="P219" s="16" t="str">
-        <x:v>V N
-V N</x:v>
+        <x:v>Verb
+Noun</x:v>
       </x:c>
     </x:row>
     <x:row r="220" ht="36" customHeight="1">
@@ -10870,8 +10870,8 @@
 unite</x:v>
       </x:c>
       <x:c r="P223" s="16" t="str">
-        <x:v>N V
-N V</x:v>
+        <x:v>Noun
+Verb</x:v>
       </x:c>
     </x:row>
     <x:row r="224" ht="36" customHeight="1">
@@ -11144,7 +11144,7 @@
 efficiently</x:v>
       </x:c>
       <x:c r="P229" s="16" t="str">
-        <x:v>N Adj
+        <x:v>Noun
 Adverb</x:v>
       </x:c>
     </x:row>
@@ -11326,8 +11326,8 @@
 regarding</x:v>
       </x:c>
       <x:c r="P233" s="16" t="str">
-        <x:v>Adv Prep
-Adv Prep</x:v>
+        <x:v>Adverb
+Preposition</x:v>
       </x:c>
     </x:row>
     <x:row r="234" ht="36" customHeight="1">
@@ -11684,8 +11684,8 @@
 involve</x:v>
       </x:c>
       <x:c r="P241" s="16" t="str">
-        <x:v>Adj V
-Adj V</x:v>
+        <x:v>Adjective
+Verb</x:v>
       </x:c>
     </x:row>
     <x:row r="242" ht="36" customHeight="1">
@@ -14010,8 +14010,8 @@
 survivor</x:v>
       </x:c>
       <x:c r="P292" s="16" t="str">
-        <x:v>N N
-N N</x:v>
+        <x:v>Noun
+Noun</x:v>
       </x:c>
     </x:row>
     <x:row r="293" ht="36" customHeight="1">
@@ -14428,8 +14428,8 @@
 retirement</x:v>
       </x:c>
       <x:c r="P301" s="16" t="str">
-        <x:v>Adj N
-Adj N</x:v>
+        <x:v>Adjective
+Noun</x:v>
       </x:c>
     </x:row>
     <x:row r="302" ht="36" customHeight="1">
@@ -15787,9 +15787,9 @@
 satisfied</x:v>
       </x:c>
       <x:c r="P331" s="16" t="str">
-        <x:v>N Adj Adj
-N Adj Adj
-N Adj Adj</x:v>
+        <x:v>Noun
+Adjective
+Adjective</x:v>
       </x:c>
     </x:row>
     <x:row r="332" ht="36" customHeight="1">
@@ -16023,9 +16023,9 @@
 relative</x:v>
       </x:c>
       <x:c r="P336" s="16" t="str">
-        <x:v>Adj N Adj
-Adj N Adj
-Adj N Adj</x:v>
+        <x:v>Adjective
+Noun
+Adjective</x:v>
       </x:c>
     </x:row>
     <x:row r="337" ht="36" customHeight="1">
@@ -22450,8 +22450,8 @@
 annoying</x:v>
       </x:c>
       <x:c r="P480" s="16" t="str">
-        <x:v>Adj Adj
-Adj Adj</x:v>
+        <x:v>Adjective
+Adjective</x:v>
       </x:c>
     </x:row>
     <x:row r="481" ht="36" customHeight="1">
@@ -22996,8 +22996,8 @@
 upload</x:v>
       </x:c>
       <x:c r="P492" s="16" t="str">
-        <x:v>V V
-V V</x:v>
+        <x:v>Verb
+Verb</x:v>
       </x:c>
     </x:row>
     <x:row r="493" ht="36" customHeight="1">
@@ -27590,8 +27590,8 @@
 correspondence</x:v>
       </x:c>
       <x:c r="P595" s="16" t="str">
-        <x:v>N N
-N N</x:v>
+        <x:v>Noun
+Noun</x:v>
       </x:c>
     </x:row>
     <x:row r="596" ht="36" customHeight="1">
@@ -30444,8 +30444,8 @@
 suspicious</x:v>
       </x:c>
       <x:c r="P659" s="16" t="str">
-        <x:v>N Adj
-N Adj</x:v>
+        <x:v>Noun
+Adjective</x:v>
       </x:c>
     </x:row>
     <x:row r="660" ht="36" customHeight="1">
@@ -32152,8 +32152,8 @@
 suspicious</x:v>
       </x:c>
       <x:c r="P697" s="16" t="str">
-        <x:v>N Adj
-N Adj</x:v>
+        <x:v>Noun
+Adjective</x:v>
       </x:c>
     </x:row>
     <x:row r="698" ht="36" customHeight="1">
@@ -35892,8 +35892,8 @@
 terrorist</x:v>
       </x:c>
       <x:c r="P781" s="16" t="str">
-        <x:v>N N, Adjective
-Phrase</x:v>
+        <x:v>Noun
+Noun, Adjective</x:v>
       </x:c>
     </x:row>
     <x:row r="782" ht="36" customHeight="1">
@@ -44857,7 +44857,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R16fac8599c9145f8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R85fee67b72fb4b42"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>